<commit_message>
feat: complete 2025-2026 literature update — notes, matrix, report
- 25 paper notes (Paper_021-Paper_045) following the existing template
- Literature_Matrix.md and .xlsx: rows P021-P045 appended (schema unchanged)
- References.bib: tan2026undcs corrected to version of record (Matters Arising)
- Reports/Literature_Update_Report.md: full update report (Task 13)
- Quality checks passed: no duplicate keys/DOIs/rows, all cited keys resolve,
  all links valid, filenames consistent

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Research/Literature_Matrix/Literature_Matrix.xlsx
+++ b/02_Research/Literature_Matrix/Literature_Matrix.xlsx
@@ -129,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -152,6 +152,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -429,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S23"/>
+  <dimension ref="A1:S48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -2495,31 +2498,2431 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" s="8"/>
-    <row r="25" ht="15.75" customHeight="1" s="8"/>
-    <row r="26" ht="15.75" customHeight="1" s="8"/>
-    <row r="27" ht="15.75" customHeight="1" s="8"/>
-    <row r="28" ht="15.75" customHeight="1" s="8"/>
-    <row r="29" ht="15.75" customHeight="1" s="8"/>
-    <row r="30" ht="15.75" customHeight="1" s="8"/>
-    <row r="31" ht="15.75" customHeight="1" s="8"/>
-    <row r="32" ht="15.75" customHeight="1" s="8"/>
-    <row r="33" ht="15.75" customHeight="1" s="8"/>
-    <row r="34" ht="15.75" customHeight="1" s="8"/>
-    <row r="35" ht="15.75" customHeight="1" s="8"/>
-    <row r="36" ht="15.75" customHeight="1" s="8"/>
-    <row r="37" ht="15.75" customHeight="1" s="8"/>
-    <row r="38" ht="15.75" customHeight="1" s="8"/>
-    <row r="39" ht="15.75" customHeight="1" s="8"/>
-    <row r="40" ht="15.75" customHeight="1" s="8"/>
-    <row r="41" ht="15.75" customHeight="1" s="8"/>
-    <row r="42" ht="15.75" customHeight="1" s="8"/>
-    <row r="43" ht="15.75" customHeight="1" s="8"/>
-    <row r="44" ht="15.75" customHeight="1" s="8"/>
-    <row r="45" ht="15.75" customHeight="1" s="8"/>
-    <row r="46" ht="15.75" customHeight="1" s="8"/>
-    <row r="47" ht="15.75" customHeight="1" s="8"/>
-    <row r="48" ht="15.75" customHeight="1" s="8"/>
+    <row r="24" ht="15.75" customHeight="1" s="8">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>P021</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>A Survey of LLM-based Agents in Medicine: How far are we from Baymax?</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>Medical LLM-based agents lack a structured overview of architectures, applications, and evaluation, and are tested on static QA rather than dynamic clinical workflows.</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>A systematic survey proposing a four-pillar architecture (profile, planning, reasoning, external capacity) and four agent paradigms mapped to clinical applications and benchmarks.</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>Yes – reviews memory-enhanced reasoning and experience bases for longitudinal continuity of care.</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>Yes – surveys task decomposition, adaptive planning, and iterative self-evolution frameworks.</t>
+        </is>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>Yes – covers CoT, ToT, ReAct-style reflection, and collaborative group reasoning.</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="inlineStr">
+        <is>
+          <t>Yes – catalogs calculators, EHR interfaces, knowledge graphs, and drug databases as agent tools.</t>
+        </is>
+      </c>
+      <c r="K24" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L24" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M24" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="inlineStr">
+        <is>
+          <t>Yes – dedicates sections to hallucination, transparency/traceability, bias (BiasMedQA), and HIPAA/GDPR privacy.</t>
+        </is>
+      </c>
+      <c r="O24" s="12" t="inlineStr">
+        <is>
+          <t>Unifying taxonomy of medical agent architectures, paradigms, benchmarks, and open challenges in one reference.</t>
+        </is>
+      </c>
+      <c r="P24" s="12" t="inlineStr">
+        <is>
+          <t>Categorizes benchmarks (static QA, workflow simulation, automated) and metrics without new empirical experiments.</t>
+        </is>
+      </c>
+      <c r="Q24" s="12" t="inlineStr">
+        <is>
+          <t>Static QA benchmarks miss dynamic workflows and verification/error-correction systems remain underdeveloped.</t>
+        </is>
+      </c>
+      <c r="R24" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S24" s="12" t="inlineStr">
+        <is>
+          <t>Supplies the architectural taxonomy and confirms thesis gaps in longitudinal evaluation, patient-timeline grounding, and first-class verification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="8">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>P022</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>MedAgentBench: A Realistic Virtual EHR Environment to Benchmark Medical LLM Agents</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>Benchmark</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>No standardized benchmark exists for evaluating LLM agent capabilities in interactive medical EHR environments.</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>A 300-task physician-authored benchmark plus a FHIR-compliant interactive EHR environment with 100 patients and over 700,000 records for pass@1 evaluation.</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>No explicit persistent memory in the baseline orchestrator, though the paper notes memory-augmented designs are possible.</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>Yes – agents must plan multi-step FHIR function-call sequences stratified by difficulty (1 to 3+ steps).</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>No explicit reasoning module; reasoning is implicit in multi-round function selection.</t>
+        </is>
+      </c>
+      <c r="J25" s="12" t="inlineStr">
+        <is>
+          <t>Yes – core task is selecting and formatting FHIR GET/POST calls with LOINC, NDC, and SNOMED codes.</t>
+        </is>
+      </c>
+      <c r="K25" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L25" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M25" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N25" s="12" t="inlineStr">
+        <is>
+          <t>Yes – adopts pass@1 for clinical error intolerance and rule-based payload sanity checks, framing trust and safety barriers.</t>
+        </is>
+      </c>
+      <c r="O25" s="12" t="inlineStr">
+        <is>
+          <t>First benchmark requiring autonomous agent interaction with a migratable FHIR EHR environment.</t>
+        </is>
+      </c>
+      <c r="P25" s="12" t="inlineStr">
+        <is>
+          <t>Task success rate (overall/query/action) at pass@1 across 12 LLMs, best Claude 3.5 Sonnet v2 at 69.67%.</t>
+        </is>
+      </c>
+      <c r="Q25" s="12" t="inlineStr">
+        <is>
+          <t>Current LLMs are not reliable medical agents, especially on record-modifying action tasks.</t>
+        </is>
+      </c>
+      <c r="R25" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S25" s="12" t="inlineStr">
+        <is>
+          <t>Provides a FHIR evaluation harness and task taxonomy for the thesis action and verification layers while motivating longitudinal ICU differentiation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="8">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>P023</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>TxAgent: An AI Agent for Therapeutic Reasoning Across a Universe of Tools</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>LLMs hallucinate, lack real-time biomedical knowledge, and cannot perform the multi-step reasoning needed for treatment selection.</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>A fine-tuned LLM agent performing multi-step white-box reasoning with goal-oriented tool selection over 211 verified biomedical tools (TOOLUNIVERSE) via a TOOLRAG retriever.</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>No persistent patient memory; relies on continuously updated external knowledge bases and in-session reasoning traces.</t>
+        </is>
+      </c>
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>Yes – generates a plan then iteratively selects tools based on objectives and prior tool feedback until FINISH.</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="inlineStr">
+        <is>
+          <t>Yes – iterative multi-step reasoning with explicit thought steps that outperform multi-round calls alone.</t>
+        </is>
+      </c>
+      <c r="J26" s="12" t="inlineStr">
+        <is>
+          <t>Yes – central focus, 211 tools built via TOOLGEN from openFDA, Open Targets, and Monarch APIs with TOOLRAG selection.</t>
+        </is>
+      </c>
+      <c r="K26" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L26" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M26" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr">
+        <is>
+          <t>Yes – transparent reasoning traces and verified-source grounding let users audit each therapeutic decision.</t>
+        </is>
+      </c>
+      <c r="O26" s="12" t="inlineStr">
+        <is>
+          <t>Real-time tool-based retrieval and TOOLRAG selection that keep an 8B agent current and robust across drug-name variants.</t>
+        </is>
+      </c>
+      <c r="P26" s="12" t="inlineStr">
+        <is>
+          <t>Five new benchmarks (3,168 drug tasks, 456 treatment scenarios); 92.1% open-ended DrugPC, beating GPT-4o and DeepSeek-R1.</t>
+        </is>
+      </c>
+      <c r="Q26" s="12" t="inlineStr">
+        <is>
+          <t>LLM knowledge obsolescence and shallow single-step tool use in therapeutic reasoning.</t>
+        </is>
+      </c>
+      <c r="R26" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="S26" s="12" t="inlineStr">
+        <is>
+          <t>Models the thesis reasoning-plus-tool-use loop with auditable traces and RAG grounding, to be extended with patient-timeline memory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="8">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>P024</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>DoctorAgent-RL: Real-World Doctor Agent with Proactive Consultation through Multi-Agent Reinforcement Learning</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>Single-turn and supervised dialogue systems cannot adapt questioning strategies under patient-led uncertainty or achieve genuine clinical reasoning.</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>A multi-agent reinforcement learning framework modeling consultation as an MDP, training a doctor agent via SFT plus GRPO against patient and evaluator agents.</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>No explicit persistent memory; state is the evolving multi-turn dialogue with a hidden patient profile revealed progressively.</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>Yes – the doctor agent learns to plan an adaptive information-gathering path across turns under a dynamic turn budget.</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="inlineStr">
+        <is>
+          <t>Yes – reasoning distillation with structured think traces plus RL-learned strategic layered questioning.</t>
+        </is>
+      </c>
+      <c r="J27" s="12" t="inlineStr">
+        <is>
+          <t>No – does not rely on external tool or API calls; intelligence lies in dialogue policy.</t>
+        </is>
+      </c>
+      <c r="K27" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M27" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N27" s="12" t="inlineStr">
+        <is>
+          <t>Yes – validated via blinded human assessment, real-patient trials, and ablations, though without a formal audit gate.</t>
+        </is>
+      </c>
+      <c r="O27" s="12" t="inlineStr">
+        <is>
+          <t>Learning a proactive questioning methodology via multi-agent RL rather than imitating static dialogue transcripts.</t>
+        </is>
+      </c>
+      <c r="P27" s="12" t="inlineStr">
+        <is>
+          <t>MTMedDialog scoring plus real-patient trials; 53.9% average, best across eight disease categories, 70% real-patient exact match.</t>
+        </is>
+      </c>
+      <c r="Q27" s="12" t="inlineStr">
+        <is>
+          <t>Prior methods cannot optimize proactive inquiry or validate in real clinical settings with uncertainty.</t>
+        </is>
+      </c>
+      <c r="R27" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="S27" s="12" t="inlineStr">
+        <is>
+          <t>Offers a proactive questioning and evaluator-reward paradigm plus real-patient validation methodology for the thesis human-in-the-loop layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1" s="8">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>P025</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>Towards Conversational AI for Disease Management</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>Management reasoning over longitudinal visits and safe prescribing is under-explored and hard to evaluate beyond diagnostic accuracy.</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>A dual-agent AMIE system pairing a fast Dialogue Agent with a long-context guideline-grounded Management Reasoning agent sharing persistent cross-visit state.</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>Yes – a modular persistent agent state (summary, differential, plan) maintained and updated across multiple visits.</t>
+        </is>
+      </c>
+      <c r="H28" s="12" t="inlineStr">
+        <is>
+          <t>Yes – the Mx Agent plans care via analyze-patient, set-goals, and draft-and-merge management-plan construction.</t>
+        </is>
+      </c>
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>Yes – chain-of-reasoning in the Dialogue Agent and long-context structured multi-document reasoning in the Mx Agent.</t>
+        </is>
+      </c>
+      <c r="J28" s="12" t="inlineStr">
+        <is>
+          <t>Yes – the Mx Agent is invoked as a tool and uses a Gecko-embedding retriever over guideline and formulary corpora.</t>
+        </is>
+      </c>
+      <c r="K28" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L28" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M28" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr">
+        <is>
+          <t>Yes – citation-constrained JSON output ties every plan item to a guideline for interpretability and traceability.</t>
+        </is>
+      </c>
+      <c r="O28" s="12" t="inlineStr">
+        <is>
+          <t>Dual-process two-agent design with citation-enforced structured generation grounded in NICE and BMJ guidelines.</t>
+        </is>
+      </c>
+      <c r="P28" s="12" t="inlineStr">
+        <is>
+          <t>Randomized blinded multi-visit OSCE vs 21 PCPs on 100 scenarios plus the RxQA benchmark; non-inferior and more precise.</t>
+        </is>
+      </c>
+      <c r="Q28" s="12" t="inlineStr">
+        <is>
+          <t>Little rigorous conversational, longitudinal evaluation of management reasoning existed before.</t>
+        </is>
+      </c>
+      <c r="R28" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S28" s="12" t="inlineStr">
+        <is>
+          <t>Provides a persistent cross-visit memory and citation-traceable structured-generation template directly supporting the thesis memory and verification layers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15.75" customHeight="1" s="8">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>P026</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Advancing Conversational Diagnostic AI with Multimodal Reasoning</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>Conversational diagnostic LLMs are text-only and cannot request or reason about multimodal artifacts (skin photos, ECGs, documents) mid-consultation.</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Multimodal AMIE, a state-aware dialogue phase-transition framework on Gemini 2.0 Flash that tracks patient state and uncertainty-driven differential diagnosis to strategically request and interpret multimodal artifacts.</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>Yes – within-consultation working memory via an evolving structured patient profile and dialogue history, but no persistent cross-visit memory.</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>Yes – state-driven dialogue planning decides phase transitions and targets next questions to fill prioritized information gaps.</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="inlineStr">
+        <is>
+          <t>Yes – uncertainty-directed clinical reasoning where intermediate DDx and patient-state outputs guide questioning and artifact-grounded explanations.</t>
+        </is>
+      </c>
+      <c r="J29" s="12" t="inlineStr">
+        <is>
+          <t>Yes – web search grounds management plans, while multimodal perception is native to the base model.</t>
+        </is>
+      </c>
+      <c r="K29" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L29" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M29" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N29" s="12" t="inlineStr">
+        <is>
+          <t>Yes – hallucination of image findings is an explicit safety metric with blinded randomized specialist evaluation and robustness testing.</t>
+        </is>
+      </c>
+      <c r="O29" s="12" t="inlineStr">
+        <is>
+          <t>First evidence that a conversational diagnostic AI can request and reason about multimodal artifacts during consultations, with a simulation environment and MUH OSCE rubric.</t>
+        </is>
+      </c>
+      <c r="P29" s="12" t="inlineStr">
+        <is>
+          <t>Randomized double-blind OSCE study of 105 scenarios and 210 consultations rated by specialists, where AMIE beat PCPs on 7 of 9 multimodal and 29 of 32 other axes plus auto-rater ablations.</t>
+        </is>
+      </c>
+      <c r="Q29" s="12" t="inlineStr">
+        <is>
+          <t>Evaluation is on simulated single-encounter actor scenarios rather than longitudinal real ICU records, with no persistent cross-visit memory or real-world clinical validation.</t>
+        </is>
+      </c>
+      <c r="R29" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S29" s="12" t="inlineStr">
+        <is>
+          <t>Template for the thesis patient-state layer and hallucination-as-metric verification design, and its lack of longitudinal memory and real-record evaluation directly motivates the MIMIC-IV-based framework.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1" s="8">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>P027</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>RiskAgent: Synergizing Language Models with Validated Tools for Evidence-Based Risk Prediction</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>Medical LLMs excel at exam QA but fail at precise calculation and evidence-based clinical risk prediction, hallucinate, and cannot cite evidence sources.</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>RiskAgent, a Decider-Executor-Reviewer multi-agent framework where a LoRA-tuned 8B LLaMA-3 collaborates with hundreds of validated MDCalc clinical calculators over a five-part environment.</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>No persistent patient memory – only a within-case historical-analysis store that the Reviewer reflects over.</t>
+        </is>
+      </c>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>Yes – the Decider plans tool selection and execution while the Reviewer triggers replanning when tool choice or parameter parsing fails.</t>
+        </is>
+      </c>
+      <c r="I30" s="12" t="inlineStr">
+        <is>
+          <t>Yes – tool-grounded evidence-based reasoning with an actor-critic-style reflection loop verifying each decision.</t>
+        </is>
+      </c>
+      <c r="J30" s="12" t="inlineStr">
+        <is>
+          <t>Yes – core contribution wraps 387 validated MDCalc calculators as callable tools with retrieval-ranking and parameter parsing.</t>
+        </is>
+      </c>
+      <c r="K30" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L30" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M30" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="inlineStr">
+        <is>
+          <t>Yes – faithfulness via grounding in validated tools, evidence-source tracing, a Reviewer verification gate, and explicit clinician-oversight requirement.</t>
+        </is>
+      </c>
+      <c r="O30" s="12" t="inlineStr">
+        <is>
+          <t>Synergizing a lightweight 8B model with broad validated-tool coverage plus the MedRisk benchmark of 12,352 risk-prediction questions.</t>
+        </is>
+      </c>
+      <c r="P30" s="12" t="inlineStr">
+        <is>
+          <t>On MedRisk it scores 78.34 percent qualitative and 76.33 percent quantitative, roughly doubling GPT-4o, with ablations, MedCalc-Bench tool learning, and MedQA-family QA generalization.</t>
+        </is>
+      </c>
+      <c r="Q30" s="12" t="inlineStr">
+        <is>
+          <t>Evaluated on curated benchmark questions rather than longitudinal real-patient ICU streams, and scope is limited to risk prediction with tool-library coverage constraints.</t>
+        </is>
+      </c>
+      <c r="R30" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S30" s="12" t="inlineStr">
+        <is>
+          <t>Direct model for the thesis tool-verification and audit-trail layer, its Reviewer maps to the verification gate, and it shows a lightweight deployable agent for privacy-sensitive ICU settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1" s="8">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>P028</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>HealthBench: Evaluating Large Language Models Towards Improved Human Health</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>Benchmark</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>Existing health LLM evaluations are not meaningful, trustworthy, or unsaturated, relying on exam-style questions poorly validated against expert judgment.</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>HealthBench, 5,000 realistic multi-turn health conversations graded by a validated model-based grader against 48,562 physician-written rubric criteria from 262 physicians, with Consensus and Hard variants.</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="inlineStr">
+        <is>
+          <t>No – conversations reach 19 turns but there is no persistent cross-conversation memory.</t>
+        </is>
+      </c>
+      <c r="H31" s="12" t="inlineStr">
+        <is>
+          <t>No explicit agentic planning is evaluated, though the context-seeking theme implicitly probes information-gathering behavior.</t>
+        </is>
+      </c>
+      <c r="I31" s="12" t="inlineStr">
+        <is>
+          <t>Yes – reasoning quality is probed indirectly and reasoning models like o3 score markedly higher at 60 percent.</t>
+        </is>
+      </c>
+      <c r="J31" s="12" t="inlineStr">
+        <is>
+          <t>No – evaluated models respond without external tools, and the model-based grader is only part of the evaluation pipeline.</t>
+        </is>
+      </c>
+      <c r="K31" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L31" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M31" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N31" s="12" t="inlineStr">
+        <is>
+          <t>Yes – trustworthiness is a design goal with grader meta-evaluation matching physician-physician agreement, negative-point harmful behaviors, and worst-case reliability analysis.</t>
+        </is>
+      </c>
+      <c r="O31" s="12" t="inlineStr">
+        <is>
+          <t>A meaningful, trustworthy, unsaturated physician-grounded rubric benchmark spanning 7 themes and 5 behavioral axes with open release.</t>
+        </is>
+      </c>
+      <c r="P31" s="12" t="inlineStr">
+        <is>
+          <t>5,000 conversations scored per criterion, showing GPT-3.5 Turbo 16 percent to o3 60 percent, HealthBench Hard capped at 32 percent, human baselines, and grader meta-evaluation.</t>
+        </is>
+      </c>
+      <c r="Q31" s="12" t="inlineStr">
+        <is>
+          <t>Evaluates single model responses without memory, tools, or multi-agent workflows and does not measure deployed workflows or downstream health outcomes.</t>
+        </is>
+      </c>
+      <c r="R31" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="S31" s="12" t="inlineStr">
+        <is>
+          <t>Provides the rubric-based physician-grounded evaluation template and grader meta-evaluation method for the thesis, while its single-response scope highlights the thesis differentiators of memory, tools, and orchestration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1" s="8">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>P029</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>From Human Memory to AI Memory: A Survey on Memory Mechanisms in the Era of LLMs</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>Prior reviews classify LLM memory only along the time dimension and no systematic survey connects human memory mechanisms to LLM-driven AI-system memory.</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>A three-dimensional taxonomy of object, form, and time yielding eight quadrants that maps human memory categories onto personal and system AI memory and derives open problems.</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>Yes – the entire paper, covering short-term and long-term, parametric and non-parametric memory with encoding, retrieval, consolidation, reflection, and forgetting operations.</t>
+        </is>
+      </c>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>Yes – treated as a memory consumer where system memory stores intermediate planning traces such as CoT and ReAct, though planning is not the subject.</t>
+        </is>
+      </c>
+      <c r="I32" s="12" t="inlineStr">
+        <is>
+          <t>Yes – reasoning is enhanced by stored CoT and ReAct traces and reflection over accumulated traces as a procedural-memory analogue.</t>
+        </is>
+      </c>
+      <c r="J32" s="12" t="inlineStr">
+        <is>
+          <t>No explicit focus – tool use is only mentioned as an agent capability whose intermediate results become system memory.</t>
+        </is>
+      </c>
+      <c r="K32" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L32" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M32" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr">
+        <is>
+          <t>No dedicated verification framework, though privacy and controlled forgetting are discussed as future challenges.</t>
+        </is>
+      </c>
+      <c r="O32" s="12" t="inlineStr">
+        <is>
+          <t>The object-form-time eight-quadrant taxonomy grounded in neuroscience, systematically bridging human and AI memory research.</t>
+        </is>
+      </c>
+      <c r="P32" s="12" t="inlineStr">
+        <is>
+          <t>Survey with no new experiments, cataloging memory systems like MemGPT and HippoRAG and benchmarks such as LOCOMO and BABILong.</t>
+        </is>
+      </c>
+      <c r="Q32" s="12" t="inlineStr">
+        <is>
+          <t>The field lacks comprehensive multimodal, streaming, shared, and self-evolving memory systems, and the survey offers no domain-specific clinical memory design guidance.</t>
+        </is>
+      </c>
+      <c r="R32" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S32" s="12" t="inlineStr">
+        <is>
+          <t>Supplies the theoretical scaffolding for the thesis persistent longitudinal patient memory, mapping the taxonomy onto patient-timeline episodic memory and motivating persisted reasoning traces for the audit trail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1" s="8">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>P030</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>A Survey of Agent Interoperability Protocols: MCP, ACP, A2A, and ANP</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>LLM agents suffer fragmented ad-hoc interoperability with no unified standard for capability discovery, context exchange, authentication, and cross-vendor coordination.</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>A comparative survey of MCP, ACP, A2A, and ANP as complementary interoperability tiers with per-protocol lifecycle security analysis and a phased adoption roadmap.</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>No core focus – only notes framework memory stores and ACP support for stateful long-running services.</t>
+        </is>
+      </c>
+      <c r="H33" s="12" t="inlineStr">
+        <is>
+          <t>No – mentions that agents plan multi-step workflows but studies the communication substrate beneath planning.</t>
+        </is>
+      </c>
+      <c r="I33" s="12" t="inlineStr">
+        <is>
+          <t>Yes – contextualizes ReAct and Reflexion as single-agent reasoning techniques that the protocols complement at the coordination layer.</t>
+        </is>
+      </c>
+      <c r="J33" s="12" t="inlineStr">
+        <is>
+          <t>Yes – MCP is framed as USB-C for AI, standardizing tool and context access beyond static function-calling registries.</t>
+        </is>
+      </c>
+      <c r="K33" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L33" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M33" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N33" s="12" t="inlineStr">
+        <is>
+          <t>Yes – substantial security focus with per-protocol lifecycle threat and mitigation analysis covering prompt injection, DID identity, mutual TLS, and access control.</t>
+        </is>
+      </c>
+      <c r="O33" s="12" t="inlineStr">
+        <is>
+          <t>First structured comparison of the four emerging agent interoperability protocols with a historical timeline and four-stage phased adoption roadmap.</t>
+        </is>
+      </c>
+      <c r="P33" s="12" t="inlineStr">
+        <is>
+          <t>Qualitative comparative analysis across architecture, discovery, messaging, session, and security dimensions with no empirical benchmark.</t>
+        </is>
+      </c>
+      <c r="Q33" s="12" t="inlineStr">
+        <is>
+          <t>Missing inter-protocol bridges, shared trust frameworks, and standardized multi-agent evaluation benchmarks, with no real deployment case studies including healthcare.</t>
+        </is>
+      </c>
+      <c r="R33" s="12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="S33" s="12" t="inlineStr">
+        <is>
+          <t>Informs the thesis multi-agent orchestration layer with MCP for auditable clinical tool invocation and A2A/ACP for specialist-agent coordination, plus security patterns for PHI-handling ICU deployment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1" s="8">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>P031</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Agentic Retrieval-Augmented Generation: A Survey on Agentic RAG</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>Static linear RAG pipelines cannot support multi-step reasoning or adaptation, and the fragmented Agentic RAG field lacks a unified taxonomy</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>A principled taxonomy of Agentic RAG architectures (agent cardinality, control, autonomy, knowledge representation) spanning single-agent routers, multi-agent, hierarchical/corrective, graph-based, and document workflows</t>
+        </is>
+      </c>
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>Yes – agents integrate short- and long-term memory, and long-term memory drift and selective retention are flagged as open challenges</t>
+        </is>
+      </c>
+      <c r="H34" s="12" t="inlineStr">
+        <is>
+          <t>Yes – planning is a core agentic pattern for task decomposition with recommended bounded horizons and stopping criteria</t>
+        </is>
+      </c>
+      <c r="I34" s="12" t="inlineStr">
+        <is>
+          <t>Yes – reflection and evaluator-optimizer loops (Self-Refine, Reflexion, corrective grading) drive iterative retrieval refinement</t>
+        </is>
+      </c>
+      <c r="J34" s="12" t="inlineStr">
+        <is>
+          <t>Yes – vector search, web search, APIs, and Text-to-SQL are core agentic tools under predefined access policies</t>
+        </is>
+      </c>
+      <c r="K34" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L34" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M34" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N34" s="12" t="inlineStr">
+        <is>
+          <t>Yes – calls for governance, human oversight, and explainability/traceability/auditability as first-class design goals</t>
+        </is>
+      </c>
+      <c r="O34" s="12" t="inlineStr">
+        <is>
+          <t>First principled taxonomy of Agentic RAG with comparative design trade-off analysis and workflow patterns</t>
+        </is>
+      </c>
+      <c r="P34" s="12" t="inlineStr">
+        <is>
+          <t>Catalogs QA-centric benchmarks (BEIR, HotpotQA, RAGBench) and criticizes their lack of process-level visibility into intermediate decisions</t>
+        </is>
+      </c>
+      <c r="Q34" s="12" t="inlineStr">
+        <is>
+          <t>No process-aware evaluation of reasoning trajectories, unresolved long-term memory management, and open safety/governance for autonomous RAG</t>
+        </is>
+      </c>
+      <c r="R34" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S34" s="12" t="inlineStr">
+        <is>
+          <t>Supplies the architectural vocabulary for the thesis retrieval layer and confirms medical RAG grounds in guidelines rather than the patient's own longitudinal timeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1" s="8">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>P032</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Multi-Agent Collaboration Mechanisms: A Survey of LLMs</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>Prior surveys treat multi-agent collaboration superficially, leaving no unified framework for how LLM agents actually coordinate toward shared goals</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>An extensible framework characterizing collaboration channels by actors, type (cooperation/competition/coopetition), structure (centralized/decentralized/hierarchical), strategy (rule/role/model-based), and coordination protocols</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>No – memory appears only as agent-level system prompts and cited memory-augmented generative agents, not a studied mechanism</t>
+        </is>
+      </c>
+      <c r="H35" s="12" t="inlineStr">
+        <is>
+          <t>Yes – task decomposition, orchestrator-built DAGs, and delegated long-term planning are treated as coordination concerns</t>
+        </is>
+      </c>
+      <c r="I35" s="12" t="inlineStr">
+        <is>
+          <t>Yes – multi-agent debate, competition, and Theory-of-Mind protocols are shown to improve factuality and strategic reasoning</t>
+        </is>
+      </c>
+      <c r="J35" s="12" t="inlineStr">
+        <is>
+          <t>No – tools are mentioned only as optional agent equipment (calculators, interpreters, APIs) without dedicated analysis</t>
+        </is>
+      </c>
+      <c r="K35" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L35" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M35" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N35" s="12" t="inlineStr">
+        <is>
+          <t>Yes – flags cascading hallucinations, overconfidence, adversarial exploitation, and deception risks but offers no operational countermeasures</t>
+        </is>
+      </c>
+      <c r="O35" s="12" t="inlineStr">
+        <is>
+          <t>A five-dimensional collaboration taxonomy with mathematical formalization unifying analysis and design of LLM-based MASs</t>
+        </is>
+      </c>
+      <c r="P35" s="12" t="inlineStr">
+        <is>
+          <t>No experiments; reviews MAS metrics (success rate, cost, collaborative efficiency) and concludes evaluations are narrow, inconsistent, and non-standardized</t>
+        </is>
+      </c>
+      <c r="Q35" s="12" t="inlineStr">
+        <is>
+          <t>Standardized MAS evaluation, containment of propagating errors, collective decision-making beyond voting, and scalability laws remain open</t>
+        </is>
+      </c>
+      <c r="R35" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="S35" s="12" t="inlineStr">
+        <is>
+          <t>Provides the taxonomy to describe the thesis's hierarchical role-based agent pipeline and documents the cascading-hallucination risk its verification gate operationalizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1" s="8">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>P033</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>Advances and Challenges in Foundation Agents: From Brain-Inspired Intelligence to Evolutionary, Collaborative, and Safe Systems</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>LLM-agent designs are ad hoc and piecemeal, lacking a unified framework integrating cognition, memory, world models, evolution, collaboration, and safety</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>A brain-inspired modular Foundation Agent framework with a formal perception-cognition-action loop over mental states (memory, world model, emotion, goal, reward) generalizing POMDPs</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>Yes – a dedicated chapter covers sensory/short/long-term memory and the full lifecycle, grading episodic memory and lifelong learning as underexplored</t>
+        </is>
+      </c>
+      <c r="H36" s="12" t="inlineStr">
+        <is>
+          <t>Yes – planning is formalized as an internal mental action rehearsed against the world model, plus agentic workflow optimization</t>
+        </is>
+      </c>
+      <c r="I36" s="12" t="inlineStr">
+        <is>
+          <t>Yes – structured vs unstructured reasoning is formalized as the executive function R mapping mental state to action</t>
+        </is>
+      </c>
+      <c r="J36" s="12" t="inlineStr">
+        <is>
+          <t>Yes – tool-based action paradigm plus tool optimization (learning, creation, effectiveness evaluation) are surveyed chapters</t>
+        </is>
+      </c>
+      <c r="K36" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L36" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M36" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N36" s="12" t="inlineStr">
+        <is>
+          <t>Yes – Part IV systematizes intrinsic/extrinsic threats, hallucination and injection attacks, superalignment, and a safety scaling law where capability outpaces safety</t>
+        </is>
+      </c>
+      <c r="O36" s="12" t="inlineStr">
+        <is>
+          <t>The most comprehensive formal brain-to-agent mapping with L1-L3 maturity grading exposing concrete research gaps</t>
+        </is>
+      </c>
+      <c r="P36" s="12" t="inlineStr">
+        <is>
+          <t>No experiments; reviews MAS task-solving benchmarks and empirical safety scaling analyses while noting absent standardized agent evaluation</t>
+        </is>
+      </c>
+      <c r="Q36" s="12" t="inlineStr">
+        <is>
+          <t>Episodic lifelong memory, continual learning without forgetting, world models, and safety mechanisms lagging capability remain open</t>
+        </is>
+      </c>
+      <c r="R36" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="S36" s="12" t="inlineStr">
+        <is>
+          <t>Legitimizes persistent longitudinal patient memory as a first-class cognitive module and its safety-scaling analysis motivates the thesis verification gate and human oversight</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1" s="8">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>P034</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>Survey on Evaluation of LLM-based Agents</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>Agent evaluation is fragmented, relies on coarse end-to-end metrics, saturates quickly, and ignores safety, robustness, and cost</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>The first comprehensive taxonomy of agent evaluation across capabilities, applications, generalist benchmarks, benchmark dimensions (data, environment, interface, metric, safety), and developer frameworks</t>
+        </is>
+      </c>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>Yes – dedicated section on episodic/semantic/procedural memory benchmarks finding weak long-range consistency and dynamic memory handling</t>
+        </is>
+      </c>
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>Yes – planning benchmarks (PlanBench, Natural Plan) show even SOTA models fail long-horizon planning</t>
+        </is>
+      </c>
+      <c r="I37" s="12" t="inlineStr">
+        <is>
+          <t>Yes – multi-step reasoning is evaluated with planning and flagged as obscured by end-to-end metrics needing trajectory-level assessment</t>
+        </is>
+      </c>
+      <c r="J37" s="12" t="inlineStr">
+        <is>
+          <t>Yes – traces tool-use evaluation from single-step function calling (ToolBench, BFCL) to multi-turn MCP-server frontier benchmarks</t>
+        </is>
+      </c>
+      <c r="K37" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L37" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M37" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N37" s="12" t="inlineStr">
+        <is>
+          <t>Yes – analyzes safety as a benchmark dimension, finds it nearly absent, and calls for guardrail metrics penalizing non-compliant task success</t>
+        </is>
+      </c>
+      <c r="O37" s="12" t="inlineStr">
+        <is>
+          <t>First systematic map of the agent-evaluation landscape with an orthogonal benchmark-dimension framework and live-benchmark trend analysis</t>
+        </is>
+      </c>
+      <c r="P37" s="12" t="inlineStr">
+        <is>
+          <t>The paper's core subject: metrics taxonomy (unit tests, state/answer match, pass^k), reference-based vs LLM-as-judge trajectory evaluation, and framework tooling</t>
+        </is>
+      </c>
+      <c r="Q37" s="12" t="inlineStr">
+        <is>
+          <t>Fine-grained trajectory evaluation, cost-efficiency metrics, safety/compliance testing, scalable automation, and LLM-vs-harness attribution are missing</t>
+        </is>
+      </c>
+      <c r="R37" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S37" s="12" t="inlineStr">
+        <is>
+          <t>Supplies the evaluation methodology vocabulary for the thesis and proves no longitudinal clinical benchmark exists, validating MIMIC-IV ICU evaluation as a genuine contribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1" s="8">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>P035</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>A Survey on Trustworthy LLM Agents: Threats and Countermeasures</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>Trustworthy AI</t>
+        </is>
+      </c>
+      <c r="E38" s="12" t="inlineStr">
+        <is>
+          <t>Adding memory, tools, environment, and inter-agent modules to LLMs expands the attack surface beyond what trustworthy-LLM research covers</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>The TrustAgent framework: a modular (intrinsic brain/memory/tool, extrinsic agent/environment/user), technique-oriented (attack/defense/evaluation), multi-dimensional taxonomy of agent trustworthiness</t>
+        </is>
+      </c>
+      <c r="G38" s="12" t="inlineStr">
+        <is>
+          <t>Yes – deepest coverage of memory threats (poisoning, privacy leakage, misuse) and defenses (detection, prompt modification, output intervention) for RAG-style stores</t>
+        </is>
+      </c>
+      <c r="H38" s="12" t="inlineStr">
+        <is>
+          <t>No – planning appears only as a tool-invocation phase exposing attack interfaces, not a studied capability</t>
+        </is>
+      </c>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>Yes – catalogs reasoning structures and shows backdoors can corrupt intermediate reasoning without changing final outputs, arguing for trace verification</t>
+        </is>
+      </c>
+      <c r="J38" s="12" t="inlineStr">
+        <is>
+          <t>Yes – analyzes tool manipulation and abuse attacks and finds defenses notably scarce beyond early guardrail agents</t>
+        </is>
+      </c>
+      <c r="K38" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L38" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M38" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N38" s="12" t="inlineStr">
+        <is>
+          <t>Yes – the paper's entire subject: safety, privacy, truthfulness, fairness, and robustness systematized per module with guardrail and multi-agent shield defenses</t>
+        </is>
+      </c>
+      <c r="O38" s="12" t="inlineStr">
+        <is>
+          <t>First modular attack-defense-evaluation taxonomy extending trustworthy LLMs to agents and MAS, including infectious inter-agent attacks</t>
+        </is>
+      </c>
+      <c r="P38" s="12" t="inlineStr">
+        <is>
+          <t>Surveys safety benchmarks (AgentHarm, R-Judge, InjecAgent, ToolEmu) and concludes memory and inter-agent trustworthiness evaluation are in their infancy</t>
+        </is>
+      </c>
+      <c r="Q38" s="12" t="inlineStr">
+        <is>
+          <t>Tool-invocation defenses, systematic memory and inter-agent evaluation, dynamic real-time assessment, and user trust calibration are open</t>
+        </is>
+      </c>
+      <c r="R38" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S38" s="12" t="inlineStr">
+        <is>
+          <t>Confirms verification and trustworthiness evaluation are immature field-wide, shows patient memory is a poisoning surface needing audited verification, and provides the guardrail-agent precedent for the thesis verifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1" s="8">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>P036</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>MedRAX: Medical Reasoning Agent for Chest X-ray</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
+        <is>
+          <t>Task-specific CXR models are fragmented and end-to-end multimodal LLMs hallucinate and cannot do multi-step diagnostic reasoning.</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="inlineStr">
+        <is>
+          <t>A training-free LLM agent that runs a ReAct loop orchestrating specialized CXR tools, plus the ChestAgentBench benchmark.</t>
+        </is>
+      </c>
+      <c r="G39" s="12" t="inlineStr">
+        <is>
+          <t>Yes – session-scoped short-term conversation memory with tool-output caching, but no longitudinal patient memory.</t>
+        </is>
+      </c>
+      <c r="H39" s="12" t="inlineStr">
+        <is>
+          <t>Yes – implicit ReAct planning decomposes queries into sequential tool-calling steps with loop control.</t>
+        </is>
+      </c>
+      <c r="I39" s="12" t="inlineStr">
+        <is>
+          <t>Yes – iterative observe-think-act reasoning with explicit traces that critically evaluate and resolve conflicting tool outputs.</t>
+        </is>
+      </c>
+      <c r="J39" s="12" t="inlineStr">
+        <is>
+          <t>Yes – structured JSON tool-calling across seven CXR tool categories with schema validation and parallel execution.</t>
+        </is>
+      </c>
+      <c r="K39" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L39" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M39" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N39" s="12" t="inlineStr">
+        <is>
+          <t>Yes – transparent reasoning traces and co-pilot framing, though it lacks uncertainty quantification.</t>
+        </is>
+      </c>
+      <c r="O39" s="12" t="inlineStr">
+        <is>
+          <t>First training-free specialized agentic framework that orchestrates heterogeneous CXR tools and beats monolithic models.</t>
+        </is>
+      </c>
+      <c r="P39" s="12" t="inlineStr">
+        <is>
+          <t>Achieves 63.1% on ChestAgentBench vs GPT-4o 56.4%, plus SOTA on CheXbench, MIMIC-CXR report generation, and SLAKE VQA.</t>
+        </is>
+      </c>
+      <c r="Q39" s="12" t="inlineStr">
+        <is>
+          <t>Evaluated on curated case-report VQA not longitudinal ICU records, with no uncertainty quantification or prospective validation.</t>
+        </is>
+      </c>
+      <c r="R39" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S39" s="12" t="inlineStr">
+        <is>
+          <t>Validates the LLM-driven ReAct tool-orchestration design and reusable tool-wrapper pattern for the thesis reasoning layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1" s="8">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>P037</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>Medical Hallucination in Foundation Models and Their Impact on Healthcare</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
+        <is>
+          <t>Trustworthy AI</t>
+        </is>
+      </c>
+      <c r="E40" s="12" t="inlineStr">
+        <is>
+          <t>Foundation models generate plausible but incorrect medical content that can alter clinical decisions and harm patients.</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>A five-cluster hallucination taxonomy plus multi-model benchmarking, physician-audited case annotation, and a clinician survey.</t>
+        </is>
+      </c>
+      <c r="G40" s="12" t="inlineStr">
+        <is>
+          <t>No – memory-based hallucination is a diagnostic category, not a memory mechanism.</t>
+        </is>
+      </c>
+      <c r="H40" s="12" t="inlineStr">
+        <is>
+          <t>No – concerns single-shot and prompted outputs, not planning agents.</t>
+        </is>
+      </c>
+      <c r="I40" s="12" t="inlineStr">
+        <is>
+          <t>Yes – reframes hallucination as a reasoning-driven failure mode where chain-of-thought reduces errors.</t>
+        </is>
+      </c>
+      <c r="J40" s="12" t="inlineStr">
+        <is>
+          <t>No – evaluates search and retrieval as mitigations, not agentic tool use.</t>
+        </is>
+      </c>
+      <c r="K40" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L40" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M40" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N40" s="12" t="inlineStr">
+        <is>
+          <t>Yes – hallucination, calibration, uncertainty, and human oversight are the paper's central concern.</t>
+        </is>
+      </c>
+      <c r="O40" s="12" t="inlineStr">
+        <is>
+          <t>First unified taxonomy plus physician-audited and survey-validated characterization of medical hallucination as reasoning-driven.</t>
+        </is>
+      </c>
+      <c r="P40" s="12" t="inlineStr">
+        <is>
+          <t>Med-HALT benchmarking (general 76.6% vs medical 51.3% hallucination-free), 20-case NEJM physician audit, and n=70 clinician survey.</t>
+        </is>
+      </c>
+      <c r="Q40" s="12" t="inlineStr">
+        <is>
+          <t>No standardized metrics or ground truth, and no longitudinal real-workflow evaluation linking hallucination to outcomes.</t>
+        </is>
+      </c>
+      <c r="R40" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="S40" s="12" t="inlineStr">
+        <is>
+          <t>Justifies the thesis verification gate and audit trail, and flags temporal/lab-extraction tasks as highest-risk for ICU monitoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1" s="8">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>P038</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>The Challenge of Uncertainty Quantification of Large Language Models in Medicine</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>Trustworthy AI</t>
+        </is>
+      </c>
+      <c r="E41" s="12" t="inlineStr">
+        <is>
+          <t>Medical LLMs must reliably quantify and communicate uncertainty, but existing methods and hidden proprietary probabilities fall short.</t>
+        </is>
+      </c>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>A conceptual eight-component UQ framework uniting probabilistic, linguistic, surrogate, calibration, and explainability methods.</t>
+        </is>
+      </c>
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>No – stresses dynamic patient data and continual learning but proposes no memory module.</t>
+        </is>
+      </c>
+      <c r="H41" s="12" t="inlineStr">
+        <is>
+          <t>No – borrows the PEAS environment framework but proposes no agentic planner.</t>
+        </is>
+      </c>
+      <c r="I41" s="12" t="inlineStr">
+        <is>
+          <t>Yes – advocates Reflective AI and clinician reasoning models (Bayesian, Pauker-Kassirer) for self-aware confidence reasoning.</t>
+        </is>
+      </c>
+      <c r="J41" s="12" t="inlineStr">
+        <is>
+          <t>No – discusses UQ and XAI methods rather than agent tool orchestration.</t>
+        </is>
+      </c>
+      <c r="K41" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L41" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M41" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N41" s="12" t="inlineStr">
+        <is>
+          <t>Yes – transparency, calibration, and routing high-uncertainty cases to humans are the throughline.</t>
+        </is>
+      </c>
+      <c r="O41" s="12" t="inlineStr">
+        <is>
+          <t>Reframes uncertainty as a design resource and gives a four-source driver taxonomy with an integrated UQ framework.</t>
+        </is>
+      </c>
+      <c r="P41" s="12" t="inlineStr">
+        <is>
+          <t>No new experiments; a literature review with two synthesis tables mapping UQ techniques to trustworthiness.</t>
+        </is>
+      </c>
+      <c r="Q41" s="12" t="inlineStr">
+        <is>
+          <t>The proposed framework is aspirational and unimplemented, with no metrics, datasets, or head-to-head evaluation.</t>
+        </is>
+      </c>
+      <c r="R41" s="12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="S41" s="12" t="inlineStr">
+        <is>
+          <t>Supplies the epistemic/aleatoric UQ tooling and human-referral rationale underpinning the thesis verification gate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1" s="8">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>P039</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>Revisiting the MIMIC-IV Benchmark: Experiments Using Language Models for Electronic Health Records</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>Benchmark</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="inlineStr">
+        <is>
+          <t>No standardized shareable text-input EHR benchmark blocks applying language models to health prediction tasks.</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>A Hugging Face MIMIC-IV benchmark object plus a six-feature-group template converting structured EHR data to text.</t>
+        </is>
+      </c>
+      <c r="G42" s="12" t="inlineStr">
+        <is>
+          <t>No – time-series features are collapsed by aggregation with no persistent memory.</t>
+        </is>
+      </c>
+      <c r="H42" s="12" t="inlineStr">
+        <is>
+          <t>No – only preprocessing and prompt choices, no agentic planning.</t>
+        </is>
+      </c>
+      <c r="I42" s="12" t="inlineStr">
+        <is>
+          <t>No – zero-shot LLMs give single binary yes/no judgments with no multi-step reasoning.</t>
+        </is>
+      </c>
+      <c r="J42" s="12" t="inlineStr">
+        <is>
+          <t>No – uses standard ML libraries as engineering tools only.</t>
+        </is>
+      </c>
+      <c r="K42" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L42" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M42" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N42" s="12" t="inlineStr">
+        <is>
+          <t>No – reproducibility aside, trust is not a focus, though unanswered-question rates hint at reliability issues.</t>
+        </is>
+      </c>
+      <c r="O42" s="12" t="inlineStr">
+        <is>
+          <t>Standardizes MIMIC-IV for text models and shows fine-tuned text models rival tabular classifiers while zero-shot LLMs fail.</t>
+        </is>
+      </c>
+      <c r="P42" s="12" t="inlineStr">
+        <is>
+          <t>Eight-model mortality-classification comparison: fine-tuned Transformers AU-ROC ~0.88 vs zero-shot LLMs ~0.50-0.61.</t>
+        </is>
+      </c>
+      <c r="Q42" s="12" t="inlineStr">
+        <is>
+          <t>Zero-shot LLMs cannot encode EHR representations, token truncation drops features, and only one task/dataset is tested.</t>
+        </is>
+      </c>
+      <c r="R42" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S42" s="12" t="inlineStr">
+        <is>
+          <t>Provides the reproducible MIMIC-IV benchmark and EHR-to-text recipe, and motivates agentic scaffolding over zero-shot prompting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1" s="8">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>P040</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>Development and Prospective Implementation of a Large Language Model based System for Early Sepsis Prediction</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="E43" s="12" t="inlineStr">
+        <is>
+          <t>Structured-data sepsis models miss unstructured note context and suffer poor precision and high false-alarm burden.</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>COMPOSER-LLM couples a structured deep-learning model with an uncertainty-gated LLM RAG differential-diagnosis tool.</t>
+        </is>
+      </c>
+      <c r="G43" s="12" t="inlineStr">
+        <is>
+          <t>No – aggregates per-encounter notes in a vector store but has no cross-encounter patient memory.</t>
+        </is>
+      </c>
+      <c r="H43" s="12" t="inlineStr">
+        <is>
+          <t>No – a fixed uncertainty-gated decision policy rather than an agentic planner.</t>
+        </is>
+      </c>
+      <c r="I43" s="12" t="inlineStr">
+        <is>
+          <t>Yes – a Bayesian likelihood calculator ranks 19 differentials from LLM-extracted signs, with the LLM as extractor not diagnostician.</t>
+        </is>
+      </c>
+      <c r="J43" s="12" t="inlineStr">
+        <is>
+          <t>Yes – the LLM extractor is a LangChain-orchestrated JSON microservice feeding Bayesian likelihood calculators.</t>
+        </is>
+      </c>
+      <c r="K43" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L43" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M43" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N43" s="12" t="inlineStr">
+        <is>
+          <t>Yes – conformal OOD rejection, uncertainty-gated invocation, per-sign justifications, and clinician chart review.</t>
+        </is>
+      </c>
+      <c r="O43" s="12" t="inlineStr">
+        <is>
+          <t>Uncertainty-gated LLM invocation with note-grounded RAG and Bayesian differential diagnosis, prospectively deployed in live EDs.</t>
+        </is>
+      </c>
+      <c r="P43" s="12" t="inlineStr">
+        <is>
+          <t>~2500 encounters: sensitivity 72.1%, PPV 52.9%, FAPH 0.0087, with similar prospective results across two EDs.</t>
+        </is>
+      </c>
+      <c r="Q43" s="12" t="inlineStr">
+        <is>
+          <t>Depends on note availability, uses a non-fine-tuned LLM at one site, and patient-outcome impact is unmeasured.</t>
+        </is>
+      </c>
+      <c r="R43" s="12" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="S43" s="12" t="inlineStr">
+        <is>
+          <t>The closest prospective ICU/ED analog, validating uncertainty-gated escalation and RAG grounded in the patient's own notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15.75" customHeight="1" s="8">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>P041</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="inlineStr">
+        <is>
+          <t>Retrieval Augmented Generation for 10 Large Language Models and its Generalizability in Assessing Medical Fitness</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="E44" s="12" t="inlineStr">
+        <is>
+          <t>Ungrounded LLMs hallucinate on complex preoperative fitness assessment and RAG generalizability across models and guideline corpora was unknown</t>
+        </is>
+      </c>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>LLM-RAG pipeline (LlamaIndex Auto-Merging Retrieval) over 35 local and 23 international guidelines tested across 10 LLMs against clinicians</t>
+        </is>
+      </c>
+      <c r="G44" s="12" t="inlineStr">
+        <is>
+          <t>No – static pre-indexed guideline corpus with no per-patient longitudinal memory</t>
+        </is>
+      </c>
+      <c r="H44" s="12" t="inlineStr">
+        <is>
+          <t>No – fixed single-shot retrieval-then-generate workflow without task decomposition</t>
+        </is>
+      </c>
+      <c r="I44" s="12" t="inlineStr">
+        <is>
+          <t>Yes – structured role-playing prompt elicits 8-component clinical assessment reasoning</t>
+        </is>
+      </c>
+      <c r="J44" s="12" t="inlineStr">
+        <is>
+          <t>No – retriever is the only tool with no general tool calling</t>
+        </is>
+      </c>
+      <c r="K44" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L44" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M44" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N44" s="12" t="inlineStr">
+        <is>
+          <t>Yes – strict hallucination-as-critical-error rule, S.C.O.R.E. safety scoring, and human-in-the-loop framing</t>
+        </is>
+      </c>
+      <c r="O44" s="12" t="inlineStr">
+        <is>
+          <t>First systematic benchmark of RAG generalizability across 10 LLMs showing GPT-4-RAG beats clinicians (96.4% vs 86.6%) while RAG worsens weak models</t>
+        </is>
+      </c>
+      <c r="P44" s="12" t="inlineStr">
+        <is>
+          <t>14 simulated ASA 1-3 scenarios with 3234 LLM and 448 human responses graded against expert-panel ground truth with Fisher tests and IRR</t>
+        </is>
+      </c>
+      <c r="Q44" s="12" t="inlineStr">
+        <is>
+          <t>RAG grounds only in guidelines not the patient timeline and evaluation uses curated vignettes not real longitudinal records</t>
+        </is>
+      </c>
+      <c r="R44" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S44" s="12" t="inlineStr">
+        <is>
+          <t>Validates the thesis RAG grounding layer and model selection while motivating extension to patient-timeline grounding and MIMIC-IV evaluation with reusable S.C.O.R.E. and hallucination metrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15.75" customHeight="1" s="8">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>P042</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>MedSentry: Understanding and Mitigating Safety Risks in Medical LLM Multi-Agent Systems</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t>Benchmark</t>
+        </is>
+      </c>
+      <c r="E45" s="12" t="inlineStr">
+        <is>
+          <t>Medical multi-agent systems are exploitable by insider dark-personality agents and architectural resilience to such threats was uncharted</t>
+        </is>
+      </c>
+      <c r="F45" s="12" t="inlineStr">
+        <is>
+          <t>MedSentry benchmark of 5000 stealthy adversarial prompts plus attack-defense pipeline over four MAS topologies with a PCDC Enforcement Agent defense</t>
+        </is>
+      </c>
+      <c r="G45" s="12" t="inlineStr">
+        <is>
+          <t>No – only the SharedPool topology's shared pool acts as common memory whose openness is the poisoning vulnerability</t>
+        </is>
+      </c>
+      <c r="H45" s="12" t="inlineStr">
+        <is>
+          <t>No – fixed per-topology discussion and debate protocols rather than dynamic planning</t>
+        </is>
+      </c>
+      <c r="I45" s="12" t="inlineStr">
+        <is>
+          <t>Yes – multi-agent debate and consensus reasoning studied with CoT and ReAct baselines showing more rounds amplify contamination</t>
+        </is>
+      </c>
+      <c r="J45" s="12" t="inlineStr">
+        <is>
+          <t>No – agents interact only via inter-agent channels without external tools</t>
+        </is>
+      </c>
+      <c r="K45" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L45" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M45" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N45" s="12" t="inlineStr">
+        <is>
+          <t>Yes – adversarial insider-threat modeling with psychometric screening and topology-aware isolation restoring near-baseline safety</t>
+        </is>
+      </c>
+      <c r="O45" s="12" t="inlineStr">
+        <is>
+          <t>First systematic comparison of insider-threat resilience across MAS topologies revealing SharedPool most vulnerable and Decentralized most robust</t>
+        </is>
+      </c>
+      <c r="P45" s="12" t="inlineStr">
+        <is>
+          <t>LCS and RS safety scores from an AMA-ethics Evaluator Agent across topologies with ablations on debate rounds agent count and token depth</t>
+        </is>
+      </c>
+      <c r="Q45" s="12" t="inlineStr">
+        <is>
+          <t>Defense validated only in simulated dialogues not real clinical workflows and audit-trail faithfulness of the enforcer is not itself evaluated</t>
+        </is>
+      </c>
+      <c r="R45" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="S45" s="12" t="inlineStr">
+        <is>
+          <t>Informs thesis orchestration topology and verification gate design as an Enforcement-Agent precedent and warns that shared patient memory needs write control and provenance purging</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1" s="8">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>P043</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="inlineStr">
+        <is>
+          <t>Unregulated Large Language Models Produce Medical Device-Like Output</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="inlineStr">
+        <is>
+          <t>Trustworthy AI</t>
+        </is>
+      </c>
+      <c r="E46" s="12" t="inlineStr">
+        <is>
+          <t>Unregulated general-purpose LLMs may emit FDA device-like clinical decision support despite disclaimers and prompt constraints</t>
+        </is>
+      </c>
+      <c r="F46" s="12" t="inlineStr">
+        <is>
+          <t>Empirical regulatory stress-test prompting GPT-4 and Llama-3 with FDA non-device instructions then escalating to emergencies and a jailbreak</t>
+        </is>
+      </c>
+      <c r="G46" s="12" t="inlineStr">
+        <is>
+          <t>No – sessions deliberately reset before each scenario</t>
+        </is>
+      </c>
+      <c r="H46" s="12" t="inlineStr">
+        <is>
+          <t>No – single-turn and short multi-turn prompt sequences only</t>
+        </is>
+      </c>
+      <c r="I46" s="12" t="inlineStr">
+        <is>
+          <t>No – classifies outputs against regulatory device criteria rather than studying reasoning mechanisms</t>
+        </is>
+      </c>
+      <c r="J46" s="12" t="inlineStr">
+        <is>
+          <t>No – off-the-shelf chat interfaces without tool integrations</t>
+        </is>
+      </c>
+      <c r="K46" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L46" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M46" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N46" s="12" t="inlineStr">
+        <is>
+          <t>Yes – demonstrates prompt-based guardrails fail and frames regulatory alignment as a technical alignment problem</t>
+        </is>
+      </c>
+      <c r="O46" s="12" t="inlineStr">
+        <is>
+          <t>First empirical proof that LLM output readily crosses the FDA device threshold with emergencies eliciting device-like output in up to 100% of responses</t>
+        </is>
+      </c>
+      <c r="P46" s="12" t="inlineStr">
+        <is>
+          <t>2 LLMs x 5 specialties x 3 request types x 2 prompt regimes x 5 repetitions with manual device-criteria scoring</t>
+        </is>
+      </c>
+      <c r="Q46" s="12" t="inlineStr">
+        <is>
+          <t>Only two LLMs and non-binding FDA guidance tested with no study of purpose-built verified human-supervised CDS deployments</t>
+        </is>
+      </c>
+      <c r="R46" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="S46" s="12" t="inlineStr">
+        <is>
+          <t>Establishes regulatory stakes for a time-critical ICU CDS agent and proves prompt-level controls insufficient thereby motivating the thesis architectural verification gate and audit trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15.75" customHeight="1" s="8">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>P044</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>Regulation of clinical Artificial Intelligence (AI) in the Age of Agents: Unconfined Non-Deterministic Clinical Software (UNDCS) systems for healthcare</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="inlineStr">
+        <is>
+          <t>Trustworthy AI</t>
+        </is>
+      </c>
+      <c r="E47" s="12" t="inlineStr">
+        <is>
+          <t>Label-driven SaMD regulation and exhaustive dataset testing fail for generalized non-deterministic LLM clinical software distributed direct to consumers</t>
+        </is>
+      </c>
+      <c r="F47" s="12" t="inlineStr">
+        <is>
+          <t>A new UNDCS regulatory category with mandated safeguards of red teaming guardrails confined RAG and agent-agent moderation</t>
+        </is>
+      </c>
+      <c r="G47" s="12" t="inlineStr">
+        <is>
+          <t>No – memory mechanisms are not discussed</t>
+        </is>
+      </c>
+      <c r="H47" s="12" t="inlineStr">
+        <is>
+          <t>No – planning components are not discussed</t>
+        </is>
+      </c>
+      <c r="I47" s="12" t="inlineStr">
+        <is>
+          <t>Yes – advocates neuro-symbolic deterministic reasoning from validated guidelines and repeated-sampling adjudication as safeguards</t>
+        </is>
+      </c>
+      <c r="J47" s="12" t="inlineStr">
+        <is>
+          <t>No – agentic digital functions noted as risk surface but tool mechanics not analyzed</t>
+        </is>
+      </c>
+      <c r="K47" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L47" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M47" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N47" s="12" t="inlineStr">
+        <is>
+          <t>Yes – entire paper is governance of hallucination-prone unconfined systems with layered defenses and manufacturer accountability</t>
+        </is>
+      </c>
+      <c r="O47" s="12" t="inlineStr">
+        <is>
+          <t>The DCS/CCS/UNDCS taxonomy and proposal of a new non-label-driven regulatory category for generative clinical AI</t>
+        </is>
+      </c>
+      <c r="P47" s="12" t="inlineStr">
+        <is>
+          <t>None – a 4-page Matters Arising commentary with no experiments proposing LLM-as-a-Judge adjudication in place of exhaustive dataset testing</t>
+        </is>
+      </c>
+      <c r="Q47" s="12" t="inlineStr">
+        <is>
+          <t>Safeguards remain concept-level with no operational protocol metrics or evaluation of the moderating agents themselves</t>
+        </is>
+      </c>
+      <c r="R47" s="12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="S47" s="12" t="inlineStr">
+        <is>
+          <t>Gives the thesis regulatory vocabulary to position its verification gate and human-in-the-loop layers as the agent-agent moderation and confinement safeguards UNDCS regulation would mandate</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15.75" customHeight="1" s="8">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>P045</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>Human-large language model collaboration in clinical medicine: a systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>Whether human+AI collaboration actually outperforms human-only or AI-only clinical workflows was untested beyond the assumption it is inherently beneficial</t>
+        </is>
+      </c>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>PRISMA 2020 meta-analysis of 10 trials comparing H+AI vs H with HKSJ random-effects models prediction intervals RoB 2 and GRADE</t>
+        </is>
+      </c>
+      <c r="G48" s="12" t="inlineStr">
+        <is>
+          <t>No – no pooled study involves persistent patient memory and longitudinal designs are only future work</t>
+        </is>
+      </c>
+      <c r="H48" s="12" t="inlineStr">
+        <is>
+          <t>No – analyzes clinician-LLM workflows rather than agent planning internals</t>
+        </is>
+      </c>
+      <c r="I48" s="12" t="inlineStr">
+        <is>
+          <t>Yes – synthesizes diagnostic reasoning outcomes and explains failure via anchoring automation bias and cognitive dissonance</t>
+        </is>
+      </c>
+      <c r="J48" s="12" t="inlineStr">
+        <is>
+          <t>No – the LLM itself is the clinician's tool with no tool-calling analysis</t>
+        </is>
+      </c>
+      <c r="K48" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L48" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M48" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N48" s="12" t="inlineStr">
+        <is>
+          <t>Yes – recommends safety-critical error metrics uncertainty disclosure de-anchoring mandatory review and audit traceability</t>
+        </is>
+      </c>
+      <c r="O48" s="12" t="inlineStr">
+        <is>
+          <t>Identifies the collaboration paradox (synergy ratio near 1 vs AI-only) and a 2x2 task complexity-structure framework for deployment</t>
+        </is>
+      </c>
+      <c r="P48" s="12" t="inlineStr">
+        <is>
+          <t>Pooled RR 1.59 for accuracy MD +4.88pp for composite scores and null time effect with prediction intervals crossing null and low-to-moderate GRADE certainty</t>
+        </is>
+      </c>
+      <c r="Q48" s="12" t="inlineStr">
+        <is>
+          <t>Evidence rests on near-clinical simulations with small k and no harmonized safety-focused core outcomes or real-workflow longitudinal trials</t>
+        </is>
+      </c>
+      <c r="R48" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S48" s="12" t="inlineStr">
+        <is>
+          <t>Grounds the thesis human-in-the-loop layer with the caveat that HITL is not a universal safeguard thereby motivating engineered verification interfaces and MIMIC-IV real-record evaluation</t>
+        </is>
+      </c>
+    </row>
     <row r="49" ht="15.75" customHeight="1" s="8"/>
     <row r="50" ht="15.75" customHeight="1" s="8"/>
     <row r="51" ht="15.75" customHeight="1" s="8"/>

</xml_diff>

<commit_message>
feat: examiner round-2 revisions + integrate longitudinal-EHR prior work (P046-P050)
</commit_message>
<xml_diff>
--- a/02_Research/Literature_Matrix/Literature_Matrix.xlsx
+++ b/02_Research/Literature_Matrix/Literature_Matrix.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S48"/>
+  <dimension ref="A1:S53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -4923,11 +4923,491 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="15.75" customHeight="1" s="8"/>
-    <row r="50" ht="15.75" customHeight="1" s="8"/>
-    <row r="51" ht="15.75" customHeight="1" s="8"/>
-    <row r="52" ht="15.75" customHeight="1" s="8"/>
-    <row r="53" ht="15.75" customHeight="1" s="8"/>
+    <row r="49" ht="15.75" customHeight="1" s="8">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>P046</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>CliCARE: Grounding Large Language Models in Clinical Guidelines for Decision Support over Longitudinal Cancer Electronic Health Records</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E49" s="12" t="inlineStr">
+        <is>
+          <t>LLMs fail at temporal reasoning over 20k+-token longitudinal cancer EHRs, hallucinate without process-oriented guideline grounding, and lack reliable evaluation</t>
+        </is>
+      </c>
+      <c r="F49" s="12" t="inlineStr">
+        <is>
+          <t>Transform EHRs into patient-specific Temporal Knowledge Graphs, align trajectories with a guideline KG via BERT matching plus LLM reranking and bootstrapped expansion, then generate grounded summaries and recommendations</t>
+        </is>
+      </c>
+      <c r="G49" s="12" t="inlineStr">
+        <is>
+          <t>Yes – patient history persisted as a temporal knowledge graph capturing long-range dependencies, though built by one-shot compression not agentic memory</t>
+        </is>
+      </c>
+      <c r="H49" s="12" t="inlineStr">
+        <is>
+          <t>No – fixed pipeline with no agentic planning, though guideline paths encode normative treatment sequences</t>
+        </is>
+      </c>
+      <c r="I49" s="12" t="inlineStr">
+        <is>
+          <t>Yes – temporal reasoning externalized into TKG structure plus zero-shot LLM reranking of clinically plausible trajectory-guideline alignments</t>
+        </is>
+      </c>
+      <c r="J49" s="12" t="inlineStr">
+        <is>
+          <t>No – fixed components (Longformer, BERT, linker, LLM) with no dynamic tool calling</t>
+        </is>
+      </c>
+      <c r="K49" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L49" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M49" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N49" s="12" t="inlineStr">
+        <is>
+          <t>Yes – guideline grounding to curb hallucination plus a three-judge ensemble validated against oncologists (Spearman ~0.7), but no per-output verification or audit trail</t>
+        </is>
+      </c>
+      <c r="O49" s="12" t="inlineStr">
+        <is>
+          <t>First framework aligning patient TKGs with a normative guideline KG for grounded longitudinal cancer decision support with expert-validated LLM judging</t>
+        </is>
+      </c>
+      <c r="P49" s="12" t="inlineStr">
+        <is>
+          <t>LLM-judge scores on CancerEHR (2,000 patients) and MIMIC-Cancer beat StandardRAG, BriefContext, MedRAG, KG2RAG, GNN-RAG (Gemini 2.5 Pro 4.976/4.965 vs 2.735/2.818), with ablations and length analysis</t>
+        </is>
+      </c>
+      <c r="Q49" s="12" t="inlineStr">
+        <is>
+          <t>Grounding is structural pre-generation compression with no recommendation-level verification, no audit trail, private primary dataset, oncology-only scope</t>
+        </is>
+      </c>
+      <c r="R49" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S49" s="12" t="inlineStr">
+        <is>
+          <t>Closest CDS-over-longitudinal-MIMIC-IV comparator; thesis borrows guideline grounding and judge validation but adds timestamp-aware retrieval, a verification gate, and measured audit trails instead of TKG compression</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" s="8">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>P047</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>Traj-CoA: Patient Trajectory Modeling via Chain-of-Agents for Lung Cancer Risk Prediction</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E50" s="12" t="inlineStr">
+        <is>
+          <t>Single LLMs cannot do temporal reasoning over 32k-128k-token noisy longitudinal EHRs due to lost-in-the-middle, and RAG loses scattered events</t>
+        </is>
+      </c>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>Chain of worker agents sequentially processes time-aware XML chunks distilling events into a shared EHRMem long-term memory, and a manager agent synthesizes summary plus memory into a zero-shot risk prediction</t>
+        </is>
+      </c>
+      <c r="G50" s="12" t="inlineStr">
+        <is>
+          <t>Yes – EHRMem stores deduplicated timestamped clinical events as a distilled timeline preventing forgetting (ablation: -1.8% AUROC without it)</t>
+        </is>
+      </c>
+      <c r="H50" s="12" t="inlineStr">
+        <is>
+          <t>No – fixed sequential worker-manager workflow driven by task prompts</t>
+        </is>
+      </c>
+      <c r="I50" s="12" t="inlineStr">
+        <is>
+          <t>Yes – progressive chunk-by-chunk temporal reasoning with global synthesis weighing recent events without discarding early history</t>
+        </is>
+      </c>
+      <c r="J50" s="12" t="inlineStr">
+        <is>
+          <t>No – no external tools; knowledge access listed as future work</t>
+        </is>
+      </c>
+      <c r="K50" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L50" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M50" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N50" s="12" t="inlineStr">
+        <is>
+          <t>No – post-hoc interpretability analyses only; authors state further validation is needed for trustworthiness</t>
+        </is>
+      </c>
+      <c r="O50" s="12" t="inlineStr">
+        <is>
+          <t>First chain-of-agents plus long-term memory system for predictive temporal reasoning over ultra-long EHRs, scaling positively to 160k tokens</t>
+        </is>
+      </c>
+      <c r="P50" s="12" t="inlineStr">
+        <is>
+          <t>Zero-shot AUROC 0.766 on 1-year lung cancer prediction beats supervised ML/DL/BERT and vanilla/RAG baselines on a 300-instance proprietary test set, with chunk-size and context-scaling sensitivity analyses</t>
+        </is>
+      </c>
+      <c r="Q50" s="12" t="inlineStr">
+        <is>
+          <t>Small single-institution single-task evaluation, record compressed sequentially rather than retrieved, no output verification, no audit trail, prompt-dependent</t>
+        </is>
+      </c>
+      <c r="R50" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="S50" s="12" t="inlineStr">
+        <is>
+          <t>Thesis borrows the persistent timestamped-timeline memory idea and time-aware chunking, but replaces sequential compression with timestamp-aware retrieval and adds recommendation verification plus measured audit trails</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15.75" customHeight="1" s="8">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>P048</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="inlineStr">
+        <is>
+          <t>TrajOnco: A Multi-Agent Framework for Temporal Reasoning over Longitudinal EHR for Multi-Cancer Early Detection</t>
+        </is>
+      </c>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E51" s="12" t="inlineStr">
+        <is>
+          <t>Multi-cancer early detection needs interpretable temporal reasoning over years-long EHRs, but supervised ML needs training/feature engineering and single-agent LLMs lose evolving signals</t>
+        </is>
+      </c>
+      <c r="F51" s="12" t="inlineStr">
+        <is>
+          <t>Training-free chain-of-agents with long-term memory over time-aware XML chunks outputs a 1-10 risk score, evidence-linked rationale, and identified events, generalizing across 15 cancers via prompt swaps</t>
+        </is>
+      </c>
+      <c r="G51" s="12" t="inlineStr">
+        <is>
+          <t>Yes – structured long-term memory of deduplicated timestamped risk factors gives the manager a global timeline and prevents over-abstraction</t>
+        </is>
+      </c>
+      <c r="H51" s="12" t="inlineStr">
+        <is>
+          <t>No – fixed sequential chain plus an engineered parallel two-stage variant, not dynamic planning</t>
+        </is>
+      </c>
+      <c r="I51" s="12" t="inlineStr">
+        <is>
+          <t>Yes – workers interpret temporal patterns and dynamically update risk; judge evaluation shows largest advantage in temporal reasoning (68% wins)</t>
+        </is>
+      </c>
+      <c r="J51" s="12" t="inlineStr">
+        <is>
+          <t>No – no tool use; subagents and agent skills proposed as future work</t>
+        </is>
+      </c>
+      <c r="K51" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L51" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M51" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N51" s="12" t="inlineStr">
+        <is>
+          <t>Yes – human fidelity evaluation found 90.27% of 113 evidence-linked events correct with an error taxonomy, but validation is one-off with no automated per-decision verification</t>
+        </is>
+      </c>
+      <c r="O51" s="12" t="inlineStr">
+        <is>
+          <t>Zero-shot multi-agent early detection across 15 cancers on 30+ health systems where architecture lets GPT-4.1-mini rival GPT-5, with population-level theme discovery</t>
+        </is>
+      </c>
+      <c r="P51" s="12" t="inlineStr">
+        <is>
+          <t>AUROC 0.64-0.80 across 15 matched 500/500 Truveta cohorts, 0.785 on lung benchmark near supervised XGBoost (0.796), LLM-judge and human fidelity evaluation, length/model/time-gap sensitivity analyses</t>
+        </is>
+      </c>
+      <c r="Q51" s="12" t="inlineStr">
+        <is>
+          <t>Structured data only, code-based outcomes without registry confirmation, residual hallucinations and lost uncertainty, no automated verification gate, record reprocessed per prediction</t>
+        </is>
+      </c>
+      <c r="R51" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="S51" s="12" t="inlineStr">
+        <is>
+          <t>Nearest precedent for measuring output faithfulness; thesis turns its one-off human fidelity check into an automated per-recommendation verification gate with measured audit trails on retrieved (not compressed) MIMIC-IV timelines</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15.75" customHeight="1" s="8">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>P049</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>TIMER: Temporal Instruction Modeling and Evaluation for Longitudinal Clinical Records</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>Benchmark</t>
+        </is>
+      </c>
+      <c r="E52" s="12" t="inlineStr">
+        <is>
+          <t>LLMs fail to reason across multi-visit patient timelines, and existing clinical instruction/evaluation data are recency-biased (55.3% of MedAlign questions target the final 25% of timelines)</t>
+        </is>
+      </c>
+      <c r="F52" s="12" t="inlineStr">
+        <is>
+          <t>Time-aware instruction tuning with timestamp-linked instruction-response pairs generated from real longitudinal EHRs, plus TIMER-Eval with controlled temporal distributions and clinician validation</t>
+        </is>
+      </c>
+      <c r="G52" s="12" t="inlineStr">
+        <is>
+          <t>No – temporal grounding is baked into model weights via tuning rather than an external longitudinal memory</t>
+        </is>
+      </c>
+      <c r="H52" s="12" t="inlineStr">
+        <is>
+          <t>No – no planning components; the contribution is training-data and evaluation methodology</t>
+        </is>
+      </c>
+      <c r="I52" s="12" t="inlineStr">
+        <is>
+          <t>Yes – targets temporal boundary adherence, trend detection, and chronological precision, with measurable gains in all three</t>
+        </is>
+      </c>
+      <c r="J52" s="12" t="inlineStr">
+        <is>
+          <t>No – models answer directly over in-context records without tools</t>
+        </is>
+      </c>
+      <c r="K52" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L52" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M52" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N52" s="12" t="inlineStr">
+        <is>
+          <t>Yes – clinician validation of generated data (95/100 relevance, 98/100 accuracy) and LLM-judge validated against human rankings (Spearman up to 0.97), but no output verification or fairness analysis</t>
+        </is>
+      </c>
+      <c r="O52" s="12" t="inlineStr">
+        <is>
+          <t>First timestamp-linked instruction-tuning method plus normalized temporal-position metric exposing recency/edge biases and proving train/eval distribution matching matters (+6.5%)</t>
+        </is>
+      </c>
+      <c r="P52" s="12" t="inlineStr">
+        <is>
+          <t>TIMER-tuned Llama-3.1-8B improves MedAlign correctness 30.69→34.32% and TIMER-Eval 45.02→48.51%, beats seven medical baselines and MedInstruct tuning by 6.3-8.45% head-to-head, replicated on Qwen</t>
+        </is>
+      </c>
+      <c r="Q52" s="12" t="inlineStr">
+        <is>
+          <t>Model-generated data may encode biases, single-institution Stanford source, no fairness/calibration analysis, temporal fidelity encouraged statistically but never enforced or traced per output</t>
+        </is>
+      </c>
+      <c r="R52" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="S52" s="12" t="inlineStr">
+        <is>
+          <t>Supplies the temporal-bias evidence and evaluation apparatus justifying the thesis's timestamp-aware retrieval; thesis differs by keeping the record external and retrievable with per-recommendation verification and audit trails instead of parametric tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15.75" customHeight="1" s="8">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>P050</t>
+        </is>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>RGAR: Recurrence Generation-augmented Retrieval for Factual-aware Medical Question Answering</t>
+        </is>
+      </c>
+      <c r="D53" s="12" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="E53" s="12" t="inlineStr">
+        <is>
+          <t>Medical RAG ignores factual knowledge in patient EHRs, concatenating whole records into queries so retrieval is diluted by irrelevant content on real-world EHR QA</t>
+        </is>
+      </c>
+      <c r="F53" s="12" t="inlineStr">
+        <is>
+          <t>Dual-end recurrent retrieval where conceptual knowledge retrieved from a corpus guides span-based factual extraction from the EHR, which iteratively refines corpus queries over two rounds without fine-tuning</t>
+        </is>
+      </c>
+      <c r="G53" s="12" t="inlineStr">
+        <is>
+          <t>No – no persistent memory; the EHR is per-question input and iteration state lives only in the updated query</t>
+        </is>
+      </c>
+      <c r="H53" s="12" t="inlineStr">
+        <is>
+          <t>No – fixed two-round recurrence schedule rather than agentic planning</t>
+        </is>
+      </c>
+      <c r="I53" s="12" t="inlineStr">
+        <is>
+          <t>Yes – supports multi-hop reasoning by interpreting numeric labs against retrieved knowledge, with rounds acting like reranking</t>
+        </is>
+      </c>
+      <c r="J53" s="12" t="inlineStr">
+        <is>
+          <t>No – retriever and extractor are fixed pipeline stages, not dynamically invoked tools</t>
+        </is>
+      </c>
+      <c r="K53" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L53" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M53" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N53" s="12" t="inlineStr">
+        <is>
+          <t>No – argues retrieval gives traceable reasoning and defers output validation to medical professionals without implementing verification</t>
+        </is>
+      </c>
+      <c r="O53" s="12" t="inlineStr">
+        <is>
+          <t>First Bloom's-taxonomy analysis of RAG separating factual from conceptual retrieval, with a recurrent factual-conceptual interaction loop needing no fine-tuning</t>
+        </is>
+      </c>
+      <c r="P53" s="12" t="inlineStr">
+        <is>
+          <t>Best average accuracy (61.04%, +11.91 over zero-shot) across MedQA-USMLE, MedMCQA, and MIMIC-IV-based EHRNoteQA, beating GAR/MedRAG/i-MedRAG; Llama-3.1-8B+RGAR (69.52%) beats RAG-enhanced GPT-3.5</t>
+        </is>
+      </c>
+      <c r="Q53" s="12" t="inlineStr">
+        <is>
+          <t>Factual extraction is temporally blind, MCQ accuracy is the only metric, no answer verification or audit trail, assumes EHR fits context, corpus-scale latency</t>
+        </is>
+      </c>
+      <c r="R53" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="S53" s="12" t="inlineStr">
+        <is>
+          <t>Validates the thesis's dual patient-record/knowledge retrieval design on MIMIC-IV data; thesis adds timestamp-aware timeline retrieval, persistent longitudinal memory, recommendation verification, and measured audit trails that RGAR lacks</t>
+        </is>
+      </c>
+    </row>
     <row r="54" ht="15.75" customHeight="1" s="8"/>
     <row r="55" ht="15.75" customHeight="1" s="8"/>
     <row r="56" ht="15.75" customHeight="1" s="8"/>

</xml_diff>